<commit_message>
update analysis and figures for final paper submission
</commit_message>
<xml_diff>
--- a/results/results_si2st.xlsx
+++ b/results/results_si2st.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephan/Sit2Stand/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C9F6F6A3-43A6-314F-A395-D3005E74E74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B152356-0D9E-4244-BAA7-7AC2816AAFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" xr2:uid="{F1991DE8-5E6C-1947-B7AF-EDD688A381C6}"/>
+    <workbookView xWindow="1360" yWindow="700" windowWidth="28040" windowHeight="17180" xr2:uid="{F1991DE8-5E6C-1947-B7AF-EDD688A381C6}"/>
   </bookViews>
   <sheets>
-    <sheet name="results_si2st" sheetId="1" r:id="rId1"/>
+    <sheet name="results_si2st (2026-06-06)" sheetId="1" r:id="rId1"/>
+    <sheet name="results_si2st (initial) (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="10">
   <si>
     <t>Row</t>
   </si>
@@ -57,7 +58,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -538,7 +539,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -942,6 +943,121 @@
         <v>5</v>
       </c>
       <c r="B2" s="1">
+        <v>59.847499999999997</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2.6560000000000001</v>
+      </c>
+      <c r="D2" s="1">
+        <v>7.1478999999999999</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1">
+        <v>69.186899999999994</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2.3668999999999998</v>
+      </c>
+      <c r="D3" s="1">
+        <v>12.16</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1">
+        <v>15.6052</v>
+      </c>
+      <c r="C4" s="1">
+        <v>-4.6486000000000001</v>
+      </c>
+      <c r="D4" s="1">
+        <v>70.120699999999999</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1">
+        <v>64.761700000000005</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2.4045000000000001</v>
+      </c>
+      <c r="D5" s="1">
+        <v>9.6531000000000002</v>
+      </c>
+      <c r="E5" s="1">
+        <v>2.5100000000000001E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1">
+        <v>8.2111999999999998</v>
+      </c>
+      <c r="C6" s="1">
+        <v>-4.0434999999999999</v>
+      </c>
+      <c r="D6" s="1">
+        <v>35.049500000000002</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.40289999999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{128992B7-2159-8F4B-B8AF-9AD290CA9D5F}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1">
         <v>90.713729437549304</v>
       </c>
       <c r="C2" s="1">

</xml_diff>